<commit_message>
feat: junta resultados modeloIntegrado 1250_365 na planilha de resumo
Adiciona colunas Custo/Gap por snapshot de tempo (3h‥24h) do modelo
integrado para a instância 00 e aba ModeloIntegrado com a progressão
completa. Script juntar_resultados.py reproduz a operação.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/alocacao/saidas_1250_40_365_2/resumo_custos.xlsx
+++ b/alocacao/saidas_1250_40_365_2/resumo_custos.xlsx
@@ -1,13 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Resultados_Custos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Resultados_Custos" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ModeloIntegrado" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -421,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S5"/>
+  <dimension ref="A1:AQ5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -430,7 +431,7 @@
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="17" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
     <col width="19" customWidth="1" min="8" max="8"/>
     <col width="32" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
@@ -443,6 +444,30 @@
     <col width="17" customWidth="1" min="17" max="17"/>
     <col width="114" customWidth="1" min="18" max="18"/>
     <col width="126" customWidth="1" min="19" max="19"/>
+    <col width="21" customWidth="1" min="20" max="20"/>
+    <col width="30" customWidth="1" min="21" max="21"/>
+    <col width="27" customWidth="1" min="22" max="22"/>
+    <col width="21" customWidth="1" min="23" max="23"/>
+    <col width="30" customWidth="1" min="24" max="24"/>
+    <col width="27" customWidth="1" min="25" max="25"/>
+    <col width="21" customWidth="1" min="26" max="26"/>
+    <col width="30" customWidth="1" min="27" max="27"/>
+    <col width="27" customWidth="1" min="28" max="28"/>
+    <col width="22" customWidth="1" min="29" max="29"/>
+    <col width="31" customWidth="1" min="30" max="30"/>
+    <col width="28" customWidth="1" min="31" max="31"/>
+    <col width="22" customWidth="1" min="32" max="32"/>
+    <col width="31" customWidth="1" min="33" max="33"/>
+    <col width="28" customWidth="1" min="34" max="34"/>
+    <col width="22" customWidth="1" min="35" max="35"/>
+    <col width="31" customWidth="1" min="36" max="36"/>
+    <col width="28" customWidth="1" min="37" max="37"/>
+    <col width="22" customWidth="1" min="38" max="38"/>
+    <col width="31" customWidth="1" min="39" max="39"/>
+    <col width="28" customWidth="1" min="40" max="40"/>
+    <col width="22" customWidth="1" min="41" max="41"/>
+    <col width="31" customWidth="1" min="42" max="42"/>
+    <col width="28" customWidth="1" min="43" max="43"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -541,6 +566,126 @@
           <t>Pasta de Saída</t>
         </is>
       </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Custo Integrado 3h</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Gap Integrado 3h vs M1D (%)</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Gap MIP Integrado 3h (%)</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Custo Integrado 6h</t>
+        </is>
+      </c>
+      <c r="X1" t="inlineStr">
+        <is>
+          <t>Gap Integrado 6h vs M1D (%)</t>
+        </is>
+      </c>
+      <c r="Y1" t="inlineStr">
+        <is>
+          <t>Gap MIP Integrado 6h (%)</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
+          <t>Custo Integrado 9h</t>
+        </is>
+      </c>
+      <c r="AA1" t="inlineStr">
+        <is>
+          <t>Gap Integrado 9h vs M1D (%)</t>
+        </is>
+      </c>
+      <c r="AB1" t="inlineStr">
+        <is>
+          <t>Gap MIP Integrado 9h (%)</t>
+        </is>
+      </c>
+      <c r="AC1" t="inlineStr">
+        <is>
+          <t>Custo Integrado 12h</t>
+        </is>
+      </c>
+      <c r="AD1" t="inlineStr">
+        <is>
+          <t>Gap Integrado 12h vs M1D (%)</t>
+        </is>
+      </c>
+      <c r="AE1" t="inlineStr">
+        <is>
+          <t>Gap MIP Integrado 12h (%)</t>
+        </is>
+      </c>
+      <c r="AF1" t="inlineStr">
+        <is>
+          <t>Custo Integrado 15h</t>
+        </is>
+      </c>
+      <c r="AG1" t="inlineStr">
+        <is>
+          <t>Gap Integrado 15h vs M1D (%)</t>
+        </is>
+      </c>
+      <c r="AH1" t="inlineStr">
+        <is>
+          <t>Gap MIP Integrado 15h (%)</t>
+        </is>
+      </c>
+      <c r="AI1" t="inlineStr">
+        <is>
+          <t>Custo Integrado 18h</t>
+        </is>
+      </c>
+      <c r="AJ1" t="inlineStr">
+        <is>
+          <t>Gap Integrado 18h vs M1D (%)</t>
+        </is>
+      </c>
+      <c r="AK1" t="inlineStr">
+        <is>
+          <t>Gap MIP Integrado 18h (%)</t>
+        </is>
+      </c>
+      <c r="AL1" t="inlineStr">
+        <is>
+          <t>Custo Integrado 21h</t>
+        </is>
+      </c>
+      <c r="AM1" t="inlineStr">
+        <is>
+          <t>Gap Integrado 21h vs M1D (%)</t>
+        </is>
+      </c>
+      <c r="AN1" t="inlineStr">
+        <is>
+          <t>Gap MIP Integrado 21h (%)</t>
+        </is>
+      </c>
+      <c r="AO1" t="inlineStr">
+        <is>
+          <t>Custo Integrado 24h</t>
+        </is>
+      </c>
+      <c r="AP1" t="inlineStr">
+        <is>
+          <t>Gap Integrado 24h vs M1D (%)</t>
+        </is>
+      </c>
+      <c r="AQ1" t="inlineStr">
+        <is>
+          <t>Gap MIP Integrado 24h (%)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
@@ -608,6 +753,78 @@
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1250_40_365_2\alocacao_abastecimento_00_1250</t>
         </is>
       </c>
+      <c r="T2" s="3" t="n">
+        <v>977233.66</v>
+      </c>
+      <c r="U2" s="4" t="n">
+        <v>7.04</v>
+      </c>
+      <c r="V2" s="4" t="n">
+        <v>11.111</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>932185.5</v>
+      </c>
+      <c r="X2" s="4" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="Y2" s="4" t="n">
+        <v>6.8154</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>928467.35</v>
+      </c>
+      <c r="AA2" s="4" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="AB2" s="4" t="n">
+        <v>6.4422</v>
+      </c>
+      <c r="AC2" s="3" t="n">
+        <v>923306.0600000001</v>
+      </c>
+      <c r="AD2" s="4" t="n">
+        <v>1.13</v>
+      </c>
+      <c r="AE2" s="4" t="n">
+        <v>5.9192</v>
+      </c>
+      <c r="AF2" s="3" t="n">
+        <v>920978.04</v>
+      </c>
+      <c r="AG2" s="4" t="n">
+        <v>0.88</v>
+      </c>
+      <c r="AH2" s="4" t="n">
+        <v>5.6814</v>
+      </c>
+      <c r="AI2" s="3" t="n">
+        <v>919099.2</v>
+      </c>
+      <c r="AJ2" s="4" t="n">
+        <v>0.67</v>
+      </c>
+      <c r="AK2" s="4" t="n">
+        <v>5.4886</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>918167.3</v>
+      </c>
+      <c r="AM2" s="4" t="n">
+        <v>0.57</v>
+      </c>
+      <c r="AN2" s="4" t="n">
+        <v>5.3927</v>
+      </c>
+      <c r="AO2" s="3" t="n">
+        <v>917814.34</v>
+      </c>
+      <c r="AP2" s="4" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="AQ2" s="4" t="n">
+        <v>5.3563</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
@@ -675,6 +892,30 @@
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1250_40_365_2\alocacao_abastecimento_10wlim_1250</t>
         </is>
       </c>
+      <c r="T3" t="inlineStr"/>
+      <c r="U3" t="inlineStr"/>
+      <c r="V3" t="inlineStr"/>
+      <c r="W3" t="inlineStr"/>
+      <c r="X3" t="inlineStr"/>
+      <c r="Y3" t="inlineStr"/>
+      <c r="Z3" t="inlineStr"/>
+      <c r="AA3" t="inlineStr"/>
+      <c r="AB3" t="inlineStr"/>
+      <c r="AC3" t="inlineStr"/>
+      <c r="AD3" t="inlineStr"/>
+      <c r="AE3" t="inlineStr"/>
+      <c r="AF3" t="inlineStr"/>
+      <c r="AG3" t="inlineStr"/>
+      <c r="AH3" t="inlineStr"/>
+      <c r="AI3" t="inlineStr"/>
+      <c r="AJ3" t="inlineStr"/>
+      <c r="AK3" t="inlineStr"/>
+      <c r="AL3" t="inlineStr"/>
+      <c r="AM3" t="inlineStr"/>
+      <c r="AN3" t="inlineStr"/>
+      <c r="AO3" t="inlineStr"/>
+      <c r="AP3" t="inlineStr"/>
+      <c r="AQ3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="inlineStr">
@@ -742,6 +983,30 @@
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1250_40_365_2\alocacao_abastecimento_full_1250</t>
         </is>
       </c>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
+      <c r="Z4" t="inlineStr"/>
+      <c r="AA4" t="inlineStr"/>
+      <c r="AB4" t="inlineStr"/>
+      <c r="AC4" t="inlineStr"/>
+      <c r="AD4" t="inlineStr"/>
+      <c r="AE4" t="inlineStr"/>
+      <c r="AF4" t="inlineStr"/>
+      <c r="AG4" t="inlineStr"/>
+      <c r="AH4" t="inlineStr"/>
+      <c r="AI4" t="inlineStr"/>
+      <c r="AJ4" t="inlineStr"/>
+      <c r="AK4" t="inlineStr"/>
+      <c r="AL4" t="inlineStr"/>
+      <c r="AM4" t="inlineStr"/>
+      <c r="AN4" t="inlineStr"/>
+      <c r="AO4" t="inlineStr"/>
+      <c r="AP4" t="inlineStr"/>
+      <c r="AQ4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -808,6 +1073,350 @@
         <is>
           <t>C:\Users\lfeli\Documents\AlocacaoCarros\ModelsAndHeristics\alocacao\saidas_1250_40_365_2\alocacao_abastecimento_limite_1250</t>
         </is>
+      </c>
+      <c r="T5" t="inlineStr"/>
+      <c r="U5" t="inlineStr"/>
+      <c r="V5" t="inlineStr"/>
+      <c r="W5" t="inlineStr"/>
+      <c r="X5" t="inlineStr"/>
+      <c r="Y5" t="inlineStr"/>
+      <c r="Z5" t="inlineStr"/>
+      <c r="AA5" t="inlineStr"/>
+      <c r="AB5" t="inlineStr"/>
+      <c r="AC5" t="inlineStr"/>
+      <c r="AD5" t="inlineStr"/>
+      <c r="AE5" t="inlineStr"/>
+      <c r="AF5" t="inlineStr"/>
+      <c r="AG5" t="inlineStr"/>
+      <c r="AH5" t="inlineStr"/>
+      <c r="AI5" t="inlineStr"/>
+      <c r="AJ5" t="inlineStr"/>
+      <c r="AK5" t="inlineStr"/>
+      <c r="AL5" t="inlineStr"/>
+      <c r="AM5" t="inlineStr"/>
+      <c r="AN5" t="inlineStr"/>
+      <c r="AO5" t="inlineStr"/>
+      <c r="AP5" t="inlineStr"/>
+      <c r="AQ5" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="21" customWidth="1" min="6" max="6"/>
+    <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>Instancia</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Hora</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Tempo_Segundos</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>Objective_HigherBound</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Best_LowerBound</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Gap_Percent</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Pico_Y</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Custo_Roteamento</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Qtd_Entregas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1250</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" t="n">
+        <v>10800</v>
+      </c>
+      <c r="D2" t="n">
+        <v>977233.6566919992</v>
+      </c>
+      <c r="E2" t="n">
+        <v>868653.1559135002</v>
+      </c>
+      <c r="F2" t="n">
+        <v>11.11100707951987</v>
+      </c>
+      <c r="G2" t="n">
+        <v>113</v>
+      </c>
+      <c r="H2" t="n">
+        <v>977233.656691991</v>
+      </c>
+      <c r="I2" t="n">
+        <v>17682</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1250</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C3" t="n">
+        <v>21600</v>
+      </c>
+      <c r="D3" t="n">
+        <v>932185.4954209998</v>
+      </c>
+      <c r="E3" t="n">
+        <v>868653.5235426745</v>
+      </c>
+      <c r="F3" t="n">
+        <v>6.815378719192858</v>
+      </c>
+      <c r="G3" t="n">
+        <v>114</v>
+      </c>
+      <c r="H3" t="n">
+        <v>932185.4954209924</v>
+      </c>
+      <c r="I3" t="n">
+        <v>17260</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1250</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>9</v>
+      </c>
+      <c r="C4" t="n">
+        <v>32400</v>
+      </c>
+      <c r="D4" t="n">
+        <v>928467.3548699998</v>
+      </c>
+      <c r="E4" t="n">
+        <v>868653.5235426745</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6.442211566576857</v>
+      </c>
+      <c r="G4" t="n">
+        <v>116</v>
+      </c>
+      <c r="H4" t="n">
+        <v>928467.3548699917</v>
+      </c>
+      <c r="I4" t="n">
+        <v>17211</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1250</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>12</v>
+      </c>
+      <c r="C5" t="n">
+        <v>43200</v>
+      </c>
+      <c r="D5" t="n">
+        <v>923306.0584769998</v>
+      </c>
+      <c r="E5" t="n">
+        <v>868653.5235426745</v>
+      </c>
+      <c r="F5" t="n">
+        <v>5.919221955986624</v>
+      </c>
+      <c r="G5" t="n">
+        <v>106</v>
+      </c>
+      <c r="H5" t="n">
+        <v>923306.0584769896</v>
+      </c>
+      <c r="I5" t="n">
+        <v>17126</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1250</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>15</v>
+      </c>
+      <c r="C6" t="n">
+        <v>54000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>920978.0371009996</v>
+      </c>
+      <c r="E6" t="n">
+        <v>868653.5235426745</v>
+      </c>
+      <c r="F6" t="n">
+        <v>5.681407313797542</v>
+      </c>
+      <c r="G6" t="n">
+        <v>110</v>
+      </c>
+      <c r="H6" t="n">
+        <v>920978.0371009884</v>
+      </c>
+      <c r="I6" t="n">
+        <v>17103</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1250</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>18</v>
+      </c>
+      <c r="C7" t="n">
+        <v>64800</v>
+      </c>
+      <c r="D7" t="n">
+        <v>919099.1993770004</v>
+      </c>
+      <c r="E7" t="n">
+        <v>868653.5235426745</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5.48859969288623</v>
+      </c>
+      <c r="G7" t="n">
+        <v>107</v>
+      </c>
+      <c r="H7" t="n">
+        <v>919099.1993769888</v>
+      </c>
+      <c r="I7" t="n">
+        <v>17072</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1250</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>21</v>
+      </c>
+      <c r="C8" t="n">
+        <v>75600</v>
+      </c>
+      <c r="D8" t="n">
+        <v>918167.302737</v>
+      </c>
+      <c r="E8" t="n">
+        <v>868653.5235426745</v>
+      </c>
+      <c r="F8" t="n">
+        <v>5.392675065505822</v>
+      </c>
+      <c r="G8" t="n">
+        <v>110</v>
+      </c>
+      <c r="H8" t="n">
+        <v>918167.3027369876</v>
+      </c>
+      <c r="I8" t="n">
+        <v>17066</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>abastecimento_00_1250</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>24</v>
+      </c>
+      <c r="C9" t="n">
+        <v>86400</v>
+      </c>
+      <c r="D9" t="n">
+        <v>917814.3425529996</v>
+      </c>
+      <c r="E9" t="n">
+        <v>868653.5235426745</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5.356292305650738</v>
+      </c>
+      <c r="G9" t="n">
+        <v>110</v>
+      </c>
+      <c r="H9" t="n">
+        <v>917814.342552988</v>
+      </c>
+      <c r="I9" t="n">
+        <v>17061</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: renomeia instancia do integrado para 'Modelo Integrado' na planilha
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/alocacao/saidas_1250_40_365_2/resumo_custos.xlsx
+++ b/alocacao/saidas_1250_40_365_2/resumo_custos.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S15"/>
+  <dimension ref="A1:S25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -609,7 +609,7 @@
       <c r="O2" s="6" t="n">
         <v>0.1565</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Q2" s="5" t="n">
@@ -676,7 +676,7 @@
       <c r="O3" s="6" t="n">
         <v>0.1609</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Q3" s="5" t="n">
@@ -743,7 +743,7 @@
       <c r="O4" s="6" t="n">
         <v>0.1669</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P4" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Q4" s="5" t="n">
@@ -810,7 +810,7 @@
       <c r="O5" s="6" t="n">
         <v>0.1568</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="Q5" s="5" t="n">
@@ -827,53 +827,83 @@
         </is>
       </c>
     </row>
-    <row r="6"/>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr"/>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr"/>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr"/>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+      <c r="S6" t="inlineStr"/>
+    </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Instancia</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
+      <c r="B7" t="inlineStr">
         <is>
           <t>Hora Limite (h)</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>Tempo Limite (s)</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>Custo Integrado</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>Gap MIP (%)</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>Custo M1 Diário (ref)</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Gap vs M1 Diário (%)</t>
         </is>
       </c>
-      <c r="H7" s="7" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>Pico Y</t>
         </is>
       </c>
-      <c r="I7" s="7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Qtd Entregas</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr"/>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr"/>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr"/>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
+      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -887,24 +917,34 @@
       <c r="C8" s="3" t="n">
         <v>10800</v>
       </c>
-      <c r="D8" s="4" t="n">
+      <c r="D8" t="n">
         <v>977233.66</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="4" t="n">
         <v>11.111</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G8" s="5" t="n">
+      <c r="G8" s="4" t="n">
         <v>7.04</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="H8" t="n">
         <v>113</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="I8" t="n">
         <v>17682</v>
       </c>
+      <c r="J8" t="inlineStr"/>
+      <c r="K8" t="inlineStr"/>
+      <c r="L8" t="inlineStr"/>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr"/>
+      <c r="O8" t="inlineStr"/>
+      <c r="P8" t="inlineStr"/>
+      <c r="Q8" t="inlineStr"/>
+      <c r="R8" t="inlineStr"/>
+      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -918,24 +958,34 @@
       <c r="C9" s="3" t="n">
         <v>21600</v>
       </c>
-      <c r="D9" s="4" t="n">
+      <c r="D9" t="n">
         <v>932185.5</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="4" t="n">
         <v>6.8154</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G9" s="5" t="n">
+      <c r="G9" s="4" t="n">
         <v>2.1</v>
       </c>
-      <c r="H9" s="3" t="n">
+      <c r="H9" t="n">
         <v>114</v>
       </c>
-      <c r="I9" s="3" t="n">
+      <c r="I9" t="n">
         <v>17260</v>
       </c>
+      <c r="J9" t="inlineStr"/>
+      <c r="K9" t="inlineStr"/>
+      <c r="L9" t="inlineStr"/>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr"/>
+      <c r="O9" t="inlineStr"/>
+      <c r="P9" t="inlineStr"/>
+      <c r="Q9" t="inlineStr"/>
+      <c r="R9" t="inlineStr"/>
+      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -949,24 +999,34 @@
       <c r="C10" s="3" t="n">
         <v>32400</v>
       </c>
-      <c r="D10" s="4" t="n">
+      <c r="D10" t="n">
         <v>928467.35</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="4" t="n">
         <v>6.4422</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G10" s="5" t="n">
+      <c r="G10" s="4" t="n">
         <v>1.7</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="H10" t="n">
         <v>116</v>
       </c>
-      <c r="I10" s="3" t="n">
+      <c r="I10" t="n">
         <v>17211</v>
       </c>
+      <c r="J10" t="inlineStr"/>
+      <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr"/>
+      <c r="O10" t="inlineStr"/>
+      <c r="P10" t="inlineStr"/>
+      <c r="Q10" t="inlineStr"/>
+      <c r="R10" t="inlineStr"/>
+      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -980,24 +1040,34 @@
       <c r="C11" s="3" t="n">
         <v>43200</v>
       </c>
-      <c r="D11" s="4" t="n">
+      <c r="D11" t="n">
         <v>923306.0600000001</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="4" t="n">
         <v>5.9192</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G11" s="5" t="n">
+      <c r="G11" s="4" t="n">
         <v>1.13</v>
       </c>
-      <c r="H11" s="3" t="n">
+      <c r="H11" t="n">
         <v>106</v>
       </c>
-      <c r="I11" s="3" t="n">
+      <c r="I11" t="n">
         <v>17126</v>
       </c>
+      <c r="J11" t="inlineStr"/>
+      <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr"/>
+      <c r="O11" t="inlineStr"/>
+      <c r="P11" t="inlineStr"/>
+      <c r="Q11" t="inlineStr"/>
+      <c r="R11" t="inlineStr"/>
+      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1011,24 +1081,34 @@
       <c r="C12" s="3" t="n">
         <v>54000</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" t="n">
         <v>920978.04</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="4" t="n">
         <v>5.6814</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="G12" s="4" t="n">
         <v>0.88</v>
       </c>
-      <c r="H12" s="3" t="n">
+      <c r="H12" t="n">
         <v>110</v>
       </c>
-      <c r="I12" s="3" t="n">
+      <c r="I12" t="n">
         <v>17103</v>
       </c>
+      <c r="J12" t="inlineStr"/>
+      <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr"/>
+      <c r="O12" t="inlineStr"/>
+      <c r="P12" t="inlineStr"/>
+      <c r="Q12" t="inlineStr"/>
+      <c r="R12" t="inlineStr"/>
+      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1042,24 +1122,34 @@
       <c r="C13" s="3" t="n">
         <v>64800</v>
       </c>
-      <c r="D13" s="4" t="n">
+      <c r="D13" t="n">
         <v>919099.2</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="4" t="n">
         <v>5.4886</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G13" s="5" t="n">
+      <c r="G13" s="4" t="n">
         <v>0.67</v>
       </c>
-      <c r="H13" s="3" t="n">
+      <c r="H13" t="n">
         <v>107</v>
       </c>
-      <c r="I13" s="3" t="n">
+      <c r="I13" t="n">
         <v>17072</v>
       </c>
+      <c r="J13" t="inlineStr"/>
+      <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr"/>
+      <c r="O13" t="inlineStr"/>
+      <c r="P13" t="inlineStr"/>
+      <c r="Q13" t="inlineStr"/>
+      <c r="R13" t="inlineStr"/>
+      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1073,24 +1163,34 @@
       <c r="C14" s="3" t="n">
         <v>75600</v>
       </c>
-      <c r="D14" s="4" t="n">
+      <c r="D14" t="n">
         <v>918167.3</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="4" t="n">
         <v>5.3927</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G14" s="5" t="n">
+      <c r="G14" s="4" t="n">
         <v>0.57</v>
       </c>
-      <c r="H14" s="3" t="n">
+      <c r="H14" t="n">
         <v>110</v>
       </c>
-      <c r="I14" s="3" t="n">
+      <c r="I14" t="n">
         <v>17066</v>
       </c>
+      <c r="J14" t="inlineStr"/>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr"/>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr"/>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1104,22 +1204,328 @@
       <c r="C15" s="3" t="n">
         <v>86400</v>
       </c>
-      <c r="D15" s="4" t="n">
+      <c r="D15" t="n">
         <v>917814.34</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="4" t="n">
         <v>5.3563</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G15" s="5" t="n">
+      <c r="G15" s="4" t="n">
         <v>0.53</v>
       </c>
-      <c r="H15" s="3" t="n">
+      <c r="H15" t="n">
         <v>110</v>
       </c>
-      <c r="I15" s="3" t="n">
+      <c r="I15" t="n">
+        <v>17061</v>
+      </c>
+      <c r="J15" t="inlineStr"/>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr"/>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr"/>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+      <c r="S15" t="inlineStr"/>
+    </row>
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>Instancia</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Hora Limite (h)</t>
+        </is>
+      </c>
+      <c r="C17" s="7" t="inlineStr">
+        <is>
+          <t>Tempo Limite (s)</t>
+        </is>
+      </c>
+      <c r="D17" s="7" t="inlineStr">
+        <is>
+          <t>Custo Integrado</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>Gap MIP (%)</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr">
+        <is>
+          <t>Custo M1 Diário (ref)</t>
+        </is>
+      </c>
+      <c r="G17" s="7" t="inlineStr">
+        <is>
+          <t>Gap vs M1 Diário (%)</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
+        <is>
+          <t>Pico Y</t>
+        </is>
+      </c>
+      <c r="I17" s="7" t="inlineStr">
+        <is>
+          <t>Qtd Entregas</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Integrado</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>10800</v>
+      </c>
+      <c r="D18" s="4" t="n">
+        <v>977233.66</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>11.111</v>
+      </c>
+      <c r="F18" s="4" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>18244465.46</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>113</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>17682</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Integrado</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>21600</v>
+      </c>
+      <c r="D19" s="4" t="n">
+        <v>932185.5</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>6.8154</v>
+      </c>
+      <c r="F19" s="4" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>17403434.16</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>114</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>17260</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Integrado</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>32400</v>
+      </c>
+      <c r="D20" s="4" t="n">
+        <v>928467.35</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>6.4422</v>
+      </c>
+      <c r="F20" s="4" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>17334017.77</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>116</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>17211</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Integrado</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>43200</v>
+      </c>
+      <c r="D21" s="4" t="n">
+        <v>923306.0600000001</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>5.9192</v>
+      </c>
+      <c r="F21" s="4" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>17237658.53</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>106</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>17126</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Integrado</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>54000</v>
+      </c>
+      <c r="D22" s="4" t="n">
+        <v>920978.04</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>5.6814</v>
+      </c>
+      <c r="F22" s="4" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>17194195.32</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>17103</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Integrado</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>64800</v>
+      </c>
+      <c r="D23" s="4" t="n">
+        <v>919099.2</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>5.4886</v>
+      </c>
+      <c r="F23" s="4" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>17159118.12</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>107</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>17072</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Integrado</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>75600</v>
+      </c>
+      <c r="D24" s="4" t="n">
+        <v>918167.3</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>5.3927</v>
+      </c>
+      <c r="F24" s="4" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>17141719.91</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>17066</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Modelo Integrado</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>86400</v>
+      </c>
+      <c r="D25" s="4" t="n">
+        <v>917814.34</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="F25" s="4" t="n">
+        <v>5.3563</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>17135130.29</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>110</v>
+      </c>
+      <c r="I25" s="3" t="n">
         <v>17061</v>
       </c>
     </row>
@@ -1137,7 +1543,7 @@
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="19" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
@@ -1198,7 +1604,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B2" s="3" t="n">
@@ -1214,10 +1620,10 @@
         <v>11.111</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>912978.58</v>
+        <v>5.3563</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>7.04</v>
+        <v>18244465.46</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>113</v>
@@ -1229,7 +1635,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
@@ -1245,10 +1651,10 @@
         <v>6.8154</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>912978.58</v>
+        <v>5.3563</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>2.1</v>
+        <v>17403434.16</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>114</v>
@@ -1260,7 +1666,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
@@ -1276,10 +1682,10 @@
         <v>6.4422</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>912978.58</v>
+        <v>5.3563</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>1.7</v>
+        <v>17334017.77</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>116</v>
@@ -1291,7 +1697,7 @@
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
@@ -1307,10 +1713,10 @@
         <v>5.9192</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>912978.58</v>
+        <v>5.3563</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>1.13</v>
+        <v>17237658.53</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>106</v>
@@ -1322,7 +1728,7 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
@@ -1338,10 +1744,10 @@
         <v>5.6814</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>912978.58</v>
+        <v>5.3563</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>0.88</v>
+        <v>17194195.32</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>110</v>
@@ -1353,7 +1759,7 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
@@ -1369,10 +1775,10 @@
         <v>5.4886</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>912978.58</v>
+        <v>5.3563</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>0.67</v>
+        <v>17159118.12</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>107</v>
@@ -1384,7 +1790,7 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -1400,10 +1806,10 @@
         <v>5.3927</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>912978.58</v>
+        <v>5.3563</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>0.57</v>
+        <v>17141719.91</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>110</v>
@@ -1415,7 +1821,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -1431,10 +1837,10 @@
         <v>5.3563</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>912978.58</v>
+        <v>5.3563</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>0.53</v>
+        <v>17135130.29</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>110</v>

</xml_diff>

<commit_message>
fix: lê backup_temporario.csv como fonte para evitar acúmulo de blocos no xlsx
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/alocacao/saidas_1250_40_365_2/resumo_custos.xlsx
+++ b/alocacao/saidas_1250_40_365_2/resumo_custos.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -588,7 +588,7 @@
       <c r="H2" s="4" t="n">
         <v>978784.13</v>
       </c>
-      <c r="I2" t="n">
+      <c r="I2" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J2" s="5" t="n">
@@ -655,7 +655,7 @@
       <c r="H3" s="4" t="n">
         <v>1052022.67</v>
       </c>
-      <c r="I3" t="n">
+      <c r="I3" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J3" s="5" t="n">
@@ -722,7 +722,7 @@
       <c r="H4" s="4" t="n">
         <v>1153077.95</v>
       </c>
-      <c r="I4" t="n">
+      <c r="I4" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J4" s="5" t="n">
@@ -789,7 +789,7 @@
       <c r="H5" s="4" t="n">
         <v>1150593.47</v>
       </c>
-      <c r="I5" t="n">
+      <c r="I5" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J5" s="5" t="n">
@@ -827,88 +827,58 @@
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" t="inlineStr"/>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-      <c r="L6" t="inlineStr"/>
-      <c r="M6" t="inlineStr"/>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
-      <c r="P6" t="inlineStr"/>
-      <c r="Q6" t="inlineStr"/>
-      <c r="R6" t="inlineStr"/>
-      <c r="S6" t="inlineStr"/>
-    </row>
+    <row r="6"/>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Instancia</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Hora Limite (h)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Tempo Limite (s)</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Custo Integrado</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Gap MIP (%)</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>Custo M1 Diário (ref)</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Gap vs M1 Diário (%)</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>Pico Y</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I7" s="7" t="inlineStr">
         <is>
           <t>Qtd Entregas</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr"/>
-      <c r="L7" t="inlineStr"/>
-      <c r="M7" t="inlineStr"/>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
@@ -917,39 +887,29 @@
       <c r="C8" s="3" t="n">
         <v>10800</v>
       </c>
-      <c r="D8" t="n">
+      <c r="D8" s="4" t="n">
         <v>977233.66</v>
       </c>
-      <c r="E8" s="4" t="n">
+      <c r="E8" s="5" t="n">
         <v>11.111</v>
       </c>
       <c r="F8" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G8" s="4" t="n">
+      <c r="G8" s="5" t="n">
         <v>7.04</v>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" s="3" t="n">
         <v>113</v>
       </c>
-      <c r="I8" t="n">
+      <c r="I8" s="3" t="n">
         <v>17682</v>
       </c>
-      <c r="J8" t="inlineStr"/>
-      <c r="K8" t="inlineStr"/>
-      <c r="L8" t="inlineStr"/>
-      <c r="M8" t="inlineStr"/>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
@@ -958,39 +918,29 @@
       <c r="C9" s="3" t="n">
         <v>21600</v>
       </c>
-      <c r="D9" t="n">
+      <c r="D9" s="4" t="n">
         <v>932185.5</v>
       </c>
-      <c r="E9" s="4" t="n">
+      <c r="E9" s="5" t="n">
         <v>6.8154</v>
       </c>
       <c r="F9" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G9" s="4" t="n">
+      <c r="G9" s="5" t="n">
         <v>2.1</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" s="3" t="n">
         <v>114</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I9" s="3" t="n">
         <v>17260</v>
       </c>
-      <c r="J9" t="inlineStr"/>
-      <c r="K9" t="inlineStr"/>
-      <c r="L9" t="inlineStr"/>
-      <c r="M9" t="inlineStr"/>
-      <c r="N9" t="inlineStr"/>
-      <c r="O9" t="inlineStr"/>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -999,39 +949,29 @@
       <c r="C10" s="3" t="n">
         <v>32400</v>
       </c>
-      <c r="D10" t="n">
+      <c r="D10" s="4" t="n">
         <v>928467.35</v>
       </c>
-      <c r="E10" s="4" t="n">
+      <c r="E10" s="5" t="n">
         <v>6.4422</v>
       </c>
       <c r="F10" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G10" s="4" t="n">
+      <c r="G10" s="5" t="n">
         <v>1.7</v>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" s="3" t="n">
         <v>116</v>
       </c>
-      <c r="I10" t="n">
+      <c r="I10" s="3" t="n">
         <v>17211</v>
       </c>
-      <c r="J10" t="inlineStr"/>
-      <c r="K10" t="inlineStr"/>
-      <c r="L10" t="inlineStr"/>
-      <c r="M10" t="inlineStr"/>
-      <c r="N10" t="inlineStr"/>
-      <c r="O10" t="inlineStr"/>
-      <c r="P10" t="inlineStr"/>
-      <c r="Q10" t="inlineStr"/>
-      <c r="R10" t="inlineStr"/>
-      <c r="S10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -1040,39 +980,29 @@
       <c r="C11" s="3" t="n">
         <v>43200</v>
       </c>
-      <c r="D11" t="n">
+      <c r="D11" s="4" t="n">
         <v>923306.0600000001</v>
       </c>
-      <c r="E11" s="4" t="n">
+      <c r="E11" s="5" t="n">
         <v>5.9192</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G11" s="4" t="n">
+      <c r="G11" s="5" t="n">
         <v>1.13</v>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" s="3" t="n">
         <v>106</v>
       </c>
-      <c r="I11" t="n">
+      <c r="I11" s="3" t="n">
         <v>17126</v>
       </c>
-      <c r="J11" t="inlineStr"/>
-      <c r="K11" t="inlineStr"/>
-      <c r="L11" t="inlineStr"/>
-      <c r="M11" t="inlineStr"/>
-      <c r="N11" t="inlineStr"/>
-      <c r="O11" t="inlineStr"/>
-      <c r="P11" t="inlineStr"/>
-      <c r="Q11" t="inlineStr"/>
-      <c r="R11" t="inlineStr"/>
-      <c r="S11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -1081,39 +1011,29 @@
       <c r="C12" s="3" t="n">
         <v>54000</v>
       </c>
-      <c r="D12" t="n">
+      <c r="D12" s="4" t="n">
         <v>920978.04</v>
       </c>
-      <c r="E12" s="4" t="n">
+      <c r="E12" s="5" t="n">
         <v>5.6814</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G12" s="4" t="n">
+      <c r="G12" s="5" t="n">
         <v>0.88</v>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="I12" t="n">
+      <c r="I12" s="3" t="n">
         <v>17103</v>
       </c>
-      <c r="J12" t="inlineStr"/>
-      <c r="K12" t="inlineStr"/>
-      <c r="L12" t="inlineStr"/>
-      <c r="M12" t="inlineStr"/>
-      <c r="N12" t="inlineStr"/>
-      <c r="O12" t="inlineStr"/>
-      <c r="P12" t="inlineStr"/>
-      <c r="Q12" t="inlineStr"/>
-      <c r="R12" t="inlineStr"/>
-      <c r="S12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -1122,39 +1042,29 @@
       <c r="C13" s="3" t="n">
         <v>64800</v>
       </c>
-      <c r="D13" t="n">
+      <c r="D13" s="4" t="n">
         <v>919099.2</v>
       </c>
-      <c r="E13" s="4" t="n">
+      <c r="E13" s="5" t="n">
         <v>5.4886</v>
       </c>
       <c r="F13" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G13" s="4" t="n">
+      <c r="G13" s="5" t="n">
         <v>0.67</v>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" s="3" t="n">
         <v>107</v>
       </c>
-      <c r="I13" t="n">
+      <c r="I13" s="3" t="n">
         <v>17072</v>
       </c>
-      <c r="J13" t="inlineStr"/>
-      <c r="K13" t="inlineStr"/>
-      <c r="L13" t="inlineStr"/>
-      <c r="M13" t="inlineStr"/>
-      <c r="N13" t="inlineStr"/>
-      <c r="O13" t="inlineStr"/>
-      <c r="P13" t="inlineStr"/>
-      <c r="Q13" t="inlineStr"/>
-      <c r="R13" t="inlineStr"/>
-      <c r="S13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -1163,39 +1073,29 @@
       <c r="C14" s="3" t="n">
         <v>75600</v>
       </c>
-      <c r="D14" t="n">
+      <c r="D14" s="4" t="n">
         <v>918167.3</v>
       </c>
-      <c r="E14" s="4" t="n">
+      <c r="E14" s="5" t="n">
         <v>5.3927</v>
       </c>
       <c r="F14" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G14" s="4" t="n">
+      <c r="G14" s="5" t="n">
         <v>0.57</v>
       </c>
-      <c r="H14" t="n">
+      <c r="H14" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="I14" t="n">
+      <c r="I14" s="3" t="n">
         <v>17066</v>
       </c>
-      <c r="J14" t="inlineStr"/>
-      <c r="K14" t="inlineStr"/>
-      <c r="L14" t="inlineStr"/>
-      <c r="M14" t="inlineStr"/>
-      <c r="N14" t="inlineStr"/>
-      <c r="O14" t="inlineStr"/>
-      <c r="P14" t="inlineStr"/>
-      <c r="Q14" t="inlineStr"/>
-      <c r="R14" t="inlineStr"/>
-      <c r="S14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>abastecimento_00_1250</t>
+          <t>Modelo Integrado</t>
         </is>
       </c>
       <c r="B15" s="3" t="n">
@@ -1204,328 +1104,22 @@
       <c r="C15" s="3" t="n">
         <v>86400</v>
       </c>
-      <c r="D15" t="n">
+      <c r="D15" s="4" t="n">
         <v>917814.34</v>
       </c>
-      <c r="E15" s="4" t="n">
+      <c r="E15" s="5" t="n">
         <v>5.3563</v>
       </c>
       <c r="F15" s="4" t="n">
         <v>912978.58</v>
       </c>
-      <c r="G15" s="4" t="n">
+      <c r="G15" s="5" t="n">
         <v>0.53</v>
       </c>
-      <c r="H15" t="n">
+      <c r="H15" s="3" t="n">
         <v>110</v>
       </c>
-      <c r="I15" t="n">
-        <v>17061</v>
-      </c>
-      <c r="J15" t="inlineStr"/>
-      <c r="K15" t="inlineStr"/>
-      <c r="L15" t="inlineStr"/>
-      <c r="M15" t="inlineStr"/>
-      <c r="N15" t="inlineStr"/>
-      <c r="O15" t="inlineStr"/>
-      <c r="P15" t="inlineStr"/>
-      <c r="Q15" t="inlineStr"/>
-      <c r="R15" t="inlineStr"/>
-      <c r="S15" t="inlineStr"/>
-    </row>
-    <row r="16"/>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
-        <is>
-          <t>Instancia</t>
-        </is>
-      </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>Hora Limite (h)</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
-        <is>
-          <t>Tempo Limite (s)</t>
-        </is>
-      </c>
-      <c r="D17" s="7" t="inlineStr">
-        <is>
-          <t>Custo Integrado</t>
-        </is>
-      </c>
-      <c r="E17" s="7" t="inlineStr">
-        <is>
-          <t>Gap MIP (%)</t>
-        </is>
-      </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>Custo M1 Diário (ref)</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Gap vs M1 Diário (%)</t>
-        </is>
-      </c>
-      <c r="H17" s="7" t="inlineStr">
-        <is>
-          <t>Pico Y</t>
-        </is>
-      </c>
-      <c r="I17" s="7" t="inlineStr">
-        <is>
-          <t>Qtd Entregas</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Modelo Integrado</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="C18" s="3" t="n">
-        <v>10800</v>
-      </c>
-      <c r="D18" s="4" t="n">
-        <v>977233.66</v>
-      </c>
-      <c r="E18" s="5" t="n">
-        <v>11.111</v>
-      </c>
-      <c r="F18" s="4" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="G18" s="5" t="n">
-        <v>18244465.46</v>
-      </c>
-      <c r="H18" s="3" t="n">
-        <v>113</v>
-      </c>
-      <c r="I18" s="3" t="n">
-        <v>17682</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>Modelo Integrado</t>
-        </is>
-      </c>
-      <c r="B19" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>21600</v>
-      </c>
-      <c r="D19" s="4" t="n">
-        <v>932185.5</v>
-      </c>
-      <c r="E19" s="5" t="n">
-        <v>6.8154</v>
-      </c>
-      <c r="F19" s="4" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="G19" s="5" t="n">
-        <v>17403434.16</v>
-      </c>
-      <c r="H19" s="3" t="n">
-        <v>114</v>
-      </c>
-      <c r="I19" s="3" t="n">
-        <v>17260</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Modelo Integrado</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="C20" s="3" t="n">
-        <v>32400</v>
-      </c>
-      <c r="D20" s="4" t="n">
-        <v>928467.35</v>
-      </c>
-      <c r="E20" s="5" t="n">
-        <v>6.4422</v>
-      </c>
-      <c r="F20" s="4" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="G20" s="5" t="n">
-        <v>17334017.77</v>
-      </c>
-      <c r="H20" s="3" t="n">
-        <v>116</v>
-      </c>
-      <c r="I20" s="3" t="n">
-        <v>17211</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Modelo Integrado</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="C21" s="3" t="n">
-        <v>43200</v>
-      </c>
-      <c r="D21" s="4" t="n">
-        <v>923306.0600000001</v>
-      </c>
-      <c r="E21" s="5" t="n">
-        <v>5.9192</v>
-      </c>
-      <c r="F21" s="4" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="G21" s="5" t="n">
-        <v>17237658.53</v>
-      </c>
-      <c r="H21" s="3" t="n">
-        <v>106</v>
-      </c>
-      <c r="I21" s="3" t="n">
-        <v>17126</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>Modelo Integrado</t>
-        </is>
-      </c>
-      <c r="B22" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="C22" s="3" t="n">
-        <v>54000</v>
-      </c>
-      <c r="D22" s="4" t="n">
-        <v>920978.04</v>
-      </c>
-      <c r="E22" s="5" t="n">
-        <v>5.6814</v>
-      </c>
-      <c r="F22" s="4" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="G22" s="5" t="n">
-        <v>17194195.32</v>
-      </c>
-      <c r="H22" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="I22" s="3" t="n">
-        <v>17103</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Modelo Integrado</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="C23" s="3" t="n">
-        <v>64800</v>
-      </c>
-      <c r="D23" s="4" t="n">
-        <v>919099.2</v>
-      </c>
-      <c r="E23" s="5" t="n">
-        <v>5.4886</v>
-      </c>
-      <c r="F23" s="4" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="G23" s="5" t="n">
-        <v>17159118.12</v>
-      </c>
-      <c r="H23" s="3" t="n">
-        <v>107</v>
-      </c>
-      <c r="I23" s="3" t="n">
-        <v>17072</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Modelo Integrado</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="C24" s="3" t="n">
-        <v>75600</v>
-      </c>
-      <c r="D24" s="4" t="n">
-        <v>918167.3</v>
-      </c>
-      <c r="E24" s="5" t="n">
-        <v>5.3927</v>
-      </c>
-      <c r="F24" s="4" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="G24" s="5" t="n">
-        <v>17141719.91</v>
-      </c>
-      <c r="H24" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="I24" s="3" t="n">
-        <v>17066</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="2" t="inlineStr">
-        <is>
-          <t>Modelo Integrado</t>
-        </is>
-      </c>
-      <c r="B25" s="3" t="n">
-        <v>24</v>
-      </c>
-      <c r="C25" s="3" t="n">
-        <v>86400</v>
-      </c>
-      <c r="D25" s="4" t="n">
-        <v>917814.34</v>
-      </c>
-      <c r="E25" s="5" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="F25" s="4" t="n">
-        <v>5.3563</v>
-      </c>
-      <c r="G25" s="5" t="n">
-        <v>17135130.29</v>
-      </c>
-      <c r="H25" s="3" t="n">
-        <v>110</v>
-      </c>
-      <c r="I25" s="3" t="n">
+      <c r="I15" s="3" t="n">
         <v>17061</v>
       </c>
     </row>
@@ -1620,10 +1214,10 @@
         <v>11.111</v>
       </c>
       <c r="F2" s="4" t="n">
-        <v>5.3563</v>
+        <v>912978.58</v>
       </c>
       <c r="G2" s="5" t="n">
-        <v>18244465.46</v>
+        <v>7.04</v>
       </c>
       <c r="H2" s="3" t="n">
         <v>113</v>
@@ -1651,10 +1245,10 @@
         <v>6.8154</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>5.3563</v>
+        <v>912978.58</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>17403434.16</v>
+        <v>2.1</v>
       </c>
       <c r="H3" s="3" t="n">
         <v>114</v>
@@ -1682,10 +1276,10 @@
         <v>6.4422</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>5.3563</v>
+        <v>912978.58</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>17334017.77</v>
+        <v>1.7</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>116</v>
@@ -1713,10 +1307,10 @@
         <v>5.9192</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>5.3563</v>
+        <v>912978.58</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>17237658.53</v>
+        <v>1.13</v>
       </c>
       <c r="H5" s="3" t="n">
         <v>106</v>
@@ -1744,10 +1338,10 @@
         <v>5.6814</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>5.3563</v>
+        <v>912978.58</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>17194195.32</v>
+        <v>0.88</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>110</v>
@@ -1775,10 +1369,10 @@
         <v>5.4886</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>5.3563</v>
+        <v>912978.58</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>17159118.12</v>
+        <v>0.67</v>
       </c>
       <c r="H7" s="3" t="n">
         <v>107</v>
@@ -1806,10 +1400,10 @@
         <v>5.3927</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>5.3563</v>
+        <v>912978.58</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>17141719.91</v>
+        <v>0.57</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>110</v>
@@ -1837,10 +1431,10 @@
         <v>5.3563</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>5.3563</v>
+        <v>912978.58</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>17135130.29</v>
+        <v>0.53</v>
       </c>
       <c r="H9" s="3" t="n">
         <v>110</v>

</xml_diff>